<commit_message>
Replace FAQ suggested answers with live agent responses; add comment column
Responses now generated directly from the AI Day Guide agent across all
30 questions. Added a yellow-tinted comment column for review feedback.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI-Day-FAQ.xlsx
+++ b/AI-Day-FAQ.xlsx
@@ -10,7 +10,7 @@
     <sheet name="FAQ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FAQ'!$A$1:$D$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FAQ'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,18 +124,15 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -500,10 +502,10 @@
   <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -519,12 +521,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Suggested answer / notes for facilitators</t>
+          <t>Agent response</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Row #</t>
+          <t>Your comments</t>
         </is>
       </c>
     </row>
@@ -538,7 +540,7 @@
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="80" customHeight="1">
       <c r="A3" s="4" t="inlineStr"/>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -547,14 +549,12 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Build something — anything — using AI. The format is open: a tool, a spec, a prototype, a game, a set of prompts. The goal is to experience building with AI and form a real opinion about it.</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
+          <t>Today you are building something — anything — using AI, and forming a real point of view on what that experience is actually like. Pick an idea (something useful, something silly, something that solves a tiny daily annoyance) and pick a surface to put it on (a receipt, a gym screen, a smart fridge, a greeting card — something unexpected). Then spend the day making it real, in whatever form makes sense to you: a prototype, a set of prompts, a spec, a piece of code, a design concept. The only rule is that you have something worth showing by the end of the day. The best way to start: tell me whether you're a researcher or a designer, and we'll get you building within five minutes.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="8" t="inlineStr"/>
       <c r="B4" s="9" t="inlineStr">
         <is>
@@ -563,14 +563,12 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Pick one idea seed (e.g. 'something that helps me make a decision I overthink') and combine it with one object (e.g. 'a gym treadmill screen'). That combination is your starting point. Don't spend more than five minutes picking.</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
+          <t>That is the right question, and I am not going to answer it for you — but I will get you there fast. Pick one idea seed from this list: something that gets you out of doing something you hate, something fun but pointless, something that helps you make a decision you always overthink, or something that makes a small moment in your day better. Now pair it with one physical object: a supermarket self-checkout, a bathroom mirror, a receipt, a museum exhibit label, a smartwatch face — anything from your everyday world. The combination is your brief. Tell me what you landed on and we will figure out what you are actually building in the next two minutes.</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="80" customHeight="1">
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -579,14 +577,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Yes. Researchers and designers have high-value roles that have nothing to do with writing code: writing specs, shaping the visual idea, evaluating what the team builds, directing the build. You can also ask Claude to write code for you without touching it yourself.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+          <t>Absolutely — and you are not at a disadvantage. Some of the most interesting things built today will not involve a single line of code: a research spec, a set of prompts, a decision aid, a design concept, a written artefact. AI is remarkably good at turning a clear idea into something tangible, and your job is to have the clear idea. The skill today is knowing what you want and being willing to push back when it is not right — that has nothing to do with coding.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="8" t="inlineStr"/>
       <c r="B6" s="9" t="inlineStr">
         <is>
@@ -595,14 +591,12 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Check the day's agenda for the exact time. As a rule: spend no more than 5 minutes picking an idea, then start building immediately. Iteration is the point — not a perfect plan upfront.</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t>I don't have the exact schedule to hand, but treat today as a full building day — likely several hours of focused time. The more important question is not how long you have total, but how quickly you can start: aim to be building something within the next five minutes, not planning what to build. Whatever you make in the first hour will be better than anything you design in your head. What are you working on?</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="80" customHeight="1">
       <c r="A7" s="4" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -611,12 +605,10 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>No. What matters is that you started, iterated at least a few times, and have a point of view on what worked and what didn't. Unfinished things make for the best debrief conversations.</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>5</v>
-      </c>
+          <t>No — you need to have something worth showing, which is different. A half-built tool with a clear point of view is more interesting than a polished thing that does nothing surprising. What matters is that you can stand up at the end of the day and say: here is what I made, here is where it worked, here is where it fell down. That is a finished thought, even if the thing itself is rough. So: start something real, and don't spend the day planning to start.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -628,7 +620,7 @@
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -637,14 +629,12 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>You have four good entry points: (1) write the spec before anyone builds, (2) shape the visual or interaction idea for builders to work from, (3) design and run an evaluation of what the team makes, or (4) build something yourself — Claude is approachable even without a coding background.</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+          <t>Your skills are exactly what today needs — framing, evaluating, writing precisely, and knowing when something is actually working. You have four real entry points: write the spec for something a designer or developer could build from, shape a visual concept using AI as your design tool, build something yourself (more possible than you might think), or run a structured evaluation of an AI tool against real research criteria. None of these are lesser options — a sharp spec or a rigorous evaluation framework is just as valuable an output as a working prototype. Pick the one that makes you lean forward, and we'll get you moving in the next five minutes.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="8" t="inlineStr"/>
       <c r="B10" s="9" t="inlineStr">
         <is>
@@ -653,14 +643,12 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Lead on the artifact itself. Your visual and experience instincts are a competitive advantage. Get to the seed-plus-object combination quickly and start iterating — trust your instincts rather than planning too much upfront.</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+          <t>Your role is to lead on the artifact itself — you own what gets made and what it looks and feels like. Today you are not just feeding prompts into a black box; you are directing, shaping, and deciding what stays and what goes. The best place to start is picking one idea seed and one object, then spending the next five minutes figuring out what you actually want to make with that combination. Once you have that, you can start building straight away — whether that is a prototype, a set of prompts, a design concept, or something that runs. What kind of thing do you want to walk away with at the end of the day?</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="80" customHeight="1">
       <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -669,14 +657,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Builders work with Claude to push the idea forward — add features, try things, fix things. Evaluators step back and ask harder questions: does this do what we said? Where does it fall down? Is AI doing the interesting work? Roles can switch. At any moment, someone should be in evaluator mode.</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+          <t>A builder makes something — a prototype, a tool, a spec, a set of prompts, anything with a shape. An evaluator takes something that exists and stress-tests it: asks where it breaks, whether it actually does what it claims, and whether AI is doing the interesting work or just the cosmetic finishing. Both are real contributions today, and they're not fixed roles — most people will shift between them as the day goes on. If you're not sure which to start as, building first usually gives you more interesting things to evaluate.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="80" customHeight="1">
       <c r="A12" s="8" t="inlineStr"/>
       <c r="B12" s="9" t="inlineStr">
         <is>
@@ -685,12 +671,10 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Yes, but it's harder. If your team is small, try switching modes deliberately — build for 20 minutes, then pause and evaluate for 5. Don't build without ever evaluating.</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>9</v>
-      </c>
+          <t>Yes, and honestly that tension is where the most interesting thinking happens. Build something, then step back and interrogate it like you didn't make it — ask where it falls down, where AI is doing real work versus just polishing. The switch between maker and critic is a skill in itself, and today is a good day to practice it. Just don't let evaluation become a way of avoiding the building part — get something made first, then tear into it.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -702,7 +686,7 @@
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="80" customHeight="1">
       <c r="A14" s="4" t="inlineStr"/>
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -711,14 +695,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Open Claude and describe what you want to make in plain language. Don't wait for a perfect prompt. The first attempt will be imperfect — that's fine. Describe what you want changed and iterate from there.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+          <t>Open a new conversation in Claude and just describe what you want to make in plain language — no special format needed. Start with one sentence: "I want to build a [thing] that [does what]." Then let Claude respond and react to what it gives you rather than trying to plan everything upfront. The fastest way to learn what works is to see something come back and disagree with it. If you have not picked what to build yet, that is the first move — not the tool.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="80" customHeight="1">
       <c r="A15" s="8" t="inlineStr"/>
       <c r="B15" s="9" t="inlineStr">
         <is>
@@ -727,14 +709,12 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Be more specific about what you want. Describe the gap between what Claude produced and what you expected. You can also ask Claude to explain what it did and why, then redirect from there.</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+          <t>Paste the prompt here and tell me what you expected to happen versus what actually happened — that gap is where the fix lives. Nine times out of ten, the issue is either that the prompt is too vague (the AI doesn't know what "good" looks like), or it's asking for too many things at once. Try splitting it: one prompt to generate, a separate prompt to refine or evaluate. If it's still off, the problem might not be the prompt — it might be that the task needs to be reframed slightly, and that's worth knowing now rather than later.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="4" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -743,14 +723,12 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Just describe what you want changed. You don't need to start over. 'Make the tone warmer', 'add a step between these two screens', 'show the result as a table instead' are all enough to go on.</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+          <t>Start by breaking what it made. Use it, find the first moment it fails or frustrates you, and tell Claude exactly what went wrong — not "make it better" but "when I do X, it does Y, and I wanted Z." That specificity is what drives a useful iteration. If Claude's output is code or a prompt, ask it to explain what it did before you change anything — that way you're editing with understanding, not guessing. Each round, hold onto what's working and name what isn't; don't let Claude rewrite the whole thing when only one part needs fixing.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="80" customHeight="1">
       <c r="A17" s="8" t="inlineStr"/>
       <c r="B17" s="9" t="inlineStr">
         <is>
@@ -759,14 +737,12 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Not during a session by default. Keep your scope tight and work with data you provide directly in the conversation. This constraint is useful — it keeps the feedback loop fast.</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+          <t>By default, Claude does not browse the internet or pull in live external data — it works from what it was trained on, with a knowledge cutoff. However, Claude can be given tools that connect it to external sources, like search APIs or databases, if someone builds that integration. For today's purposes, treat Claude as very knowledgeable but frozen in time, and plan your build around that. If your idea depends on live data — current prices, today's news, real-time anything — that is worth flagging now so you can adjust the concept before you get too far in.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="80" customHeight="1">
       <c r="A18" s="4" t="inlineStr"/>
       <c r="B18" s="5" t="inlineStr">
         <is>
@@ -775,14 +751,12 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Yes. Make sure 'Code execution and file creation' is enabled in Settings &gt; Capabilities. Claude can write, run, and iterate on code directly in the conversation.</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+          <t>Yes — Claude can write code in almost any language, and in this environment (Claude Code) it can actually run that code too, not just generate it. That means you can ask it to build something, run it, see what breaks, and iterate. For today, that opens up a lot: a working tool, a script that processes data, a simple web page, a game. The practical limit is not the language — it is having a clear enough idea of what you want to build. What are you thinking of making?</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="80" customHeight="1">
       <c r="A19" s="8" t="inlineStr"/>
       <c r="B19" s="9" t="inlineStr">
         <is>
@@ -791,12 +765,10 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Interactive tools and calculators, decision aids, games, prototypes of interfaces or flows, research specs, evaluation frameworks, sets of prompts designed for a task, visualisations, written artefacts like briefs or scripts.</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>15</v>
-      </c>
+          <t>Claude is genuinely good at things that involve language, judgment, and transformation — turning a messy input into a structured output, asking someone the right questions, explaining something complex in plain terms, or helping someone think through a decision. It works well when the "interesting work" is reasoning or writing, not pixel-perfect UI or real-time data. Concretely: decision aids that ask you a few questions and give you a recommendation, tools that reframe or summarise something, interactive prompts that feel like a conversation, and generators that take a simple input and produce something surprising. The sweet spot today is something small enough to finish, interesting enough to show — pick your seed and object and start there.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -808,7 +780,7 @@
       <c r="C20" s="3" t="inlineStr"/>
       <c r="D20" s="3" t="inlineStr"/>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21" ht="80" customHeight="1">
       <c r="A21" s="4" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -817,14 +789,12 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Set up a shared GitHub repository. One person creates it, invites the team as collaborators, and everyone clones it locally using Claude Code. Use git pull before starting work and git push to share changes.</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+          <t>The intended method is a shared GitHub repository — one person creates it, everyone else gets added as a collaborator, and each of you clones it into Claude Code on your own machine. When you've made progress on something, you push it up; your teammates pull it down. The setup guide is in the repo at github-collab-setup.md if you want the step-by-step. If GitHub feels like too much overhead right now, you can also just screenshot or export your work and drop it into a shared folder or Slack — what matters is that you have something to show at the end, not how it gets there.</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="80" customHeight="1">
       <c r="A22" s="8" t="inlineStr"/>
       <c r="B22" s="9" t="inlineStr">
         <is>
@@ -833,14 +803,12 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Create free accounts at github.com. The setup takes about five minutes. Ask a facilitator if you get stuck during account creation.</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1">
+          <t>GitHub is not required for today — it's just one way to share or collaborate on code. If you're building something that isn't code, you don't need it at all. If you are writing code, you can keep it local, paste it into a shared doc, or use something like a Replit or CodePen link to show others. Focus on what you're building, not how it's stored — you can sort sharing out at the end when you know what you've got.</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="80" customHeight="1">
       <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
@@ -849,14 +817,12 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Paste the conflict into Claude and ask it to help you resolve it. Git conflicts are clearly marked and Claude is good at walking through them.</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1">
+          <t>Open the file and look for the conflict markers — the lines starting with `&lt;&lt;&lt;&lt;&lt;&lt;&lt;`, `=======`, and `&gt;&gt;&gt;&gt;&gt;&gt;&gt;`. Everything between `&lt;&lt;&lt;&lt;&lt;&lt;&lt;` and `=======` is your version; everything between `=======` and `&gt;&gt;&gt;&gt;&gt;&gt;&gt;` is theirs. Decide together which parts to keep (often it's both, merged), delete the markers, and save. Then stage the file with `git add` and commit. If you're not using git, just paste both versions into Claude and ask it to merge them — describe which bits matter most and let it do the reconciliation.</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="80" customHeight="1">
       <c r="A24" s="8" t="inlineStr"/>
       <c r="B24" s="9" t="inlineStr">
         <is>
@@ -865,12 +831,10 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Yes. Use separate folders in your shared repo, or separate Claude conversations. Coordinate briefly so you're not duplicating effort — but parallel exploration is often valuable.</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="n">
-        <v>19</v>
-      </c>
+          <t>Absolutely — there is no rule that says a team has to build one thing together. Working in parallel is actually one of the best ways to spend the day, because you end up with multiple bets and a much richer conversation at the show-and-tell. The only thing to watch is that people do not spend so long deciding what to build separately that they lose time actually building. Split, commit to something, and check back in with each other around midday to see what is emerging.</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -882,7 +846,7 @@
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr"/>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="80" customHeight="1">
       <c r="A26" s="4" t="inlineStr"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
@@ -891,14 +855,12 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Ask: does it actually do what we said it would? Where does it fall down? Is AI doing the interesting work, or just the finishing? What would break if you removed AI entirely? Try it with at least five different inputs and notice what breaks.</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" ht="60" customHeight="1">
+          <t>Start with the bluntest test: does it actually do what you said it would do? Not in theory — run it, watch it, and be honest about where it wobbles. Then ask whether AI is doing the interesting work, or just tidying up something you could have done yourself in five minutes. The most revealing question is this one: what breaks if you remove the AI entirely? If the answer is "not much," that tells you something worth saying out loud at the showcase.</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="80" customHeight="1">
       <c r="A27" s="8" t="inlineStr"/>
       <c r="B27" s="9" t="inlineStr">
         <is>
@@ -907,14 +869,12 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Define this before you test. Ask: what would a good response look like? What would a bad one look like? Write those criteria down — that's the start of an evaluation framework. Then test against it.</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1">
+          <t>A good AI output does the actual job — it's accurate, specific enough to be useful, and doesn't require you to heavily rewrite or correct it before it's usable. A bad one is plausible-sounding but vague, confidently wrong, or generic in a way that fits any situation but none in particular. The most useful test is simple: would you show this to someone without editing it first? If the answer is yes, it earned its keep. If you spent more time fixing it than you would have spent just doing it yourself, the AI wasn't helping — it was generating work.</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28" ht="80" customHeight="1">
       <c r="A28" s="4" t="inlineStr"/>
       <c r="B28" s="5" t="inlineStr">
         <is>
@@ -923,14 +883,12 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Pause and ask: are we adding this because the thing needs it, or because we can? If it's the latter, stop. Scope creep is the most common way to end up with something you can't explain at the debrief.</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
+          <t>It is not bad by default, but it is worth pausing to ask why. Are you adding features because the thing genuinely needs them to work, or because building has momentum and it feels productive? The honest test: remove the last feature you added and see if the core idea still holds up — if it does, you might not need it. The best version of what you are making is usually the smallest version that actually does the thing.</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="80" customHeight="1">
       <c r="A29" s="8" t="inlineStr"/>
       <c r="B29" s="9" t="inlineStr">
         <is>
@@ -939,12 +897,10 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Design it like a quick usability test: define what good looks like, pick 5–10 test inputs, run them, note where the output falls short. Researchers are well-placed to lead this.</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n">
-        <v>23</v>
-      </c>
+          <t>Pick your thing first, build a version of it, then turn the evaluation questions on it like a lens — not all at once, just the ones that sting. The most useful ones are: does it actually do what you said it would do, and what would break if you removed AI entirely? Those two questions tend to expose whether AI is doing real work or just window dressing. Run it with one other person if you can — watch where they get confused or where the thing surprises them. That's your evaluation. You don't need a framework, you need honesty.</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -956,7 +912,7 @@
       <c r="C30" s="3" t="inlineStr"/>
       <c r="D30" s="3" t="inlineStr"/>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31" ht="80" customHeight="1">
       <c r="A31" s="4" t="inlineStr"/>
       <c r="B31" s="5" t="inlineStr">
         <is>
@@ -965,14 +921,12 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Any format works — a live demo, a screenshot, a file, a link, or just talking through it. There's no required format for sharing. Bring whatever exists, even if it's unfinished.</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" ht="60" customHeight="1">
+          <t>At the end of the day there will be a show-and-tell — each group gets a few minutes to share what they built and, more importantly, what they learned from building it. You do not need a polished demo. A screenshot, a walkthrough, or even just talking through what you made and where it surprised you is completely valid. The most interesting part is usually the honest answer to "where did it fall down?" — so start thinking about that now as you build. If your thing works, show it working. If it broke in an interesting way, show that too.</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="80" customHeight="1">
       <c r="A32" s="8" t="inlineStr"/>
       <c r="B32" s="9" t="inlineStr">
         <is>
@@ -981,14 +935,12 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Yes. Unfinished things often make for the most interesting debrief conversations. Explain what you tried, where you got stuck, and what you'd do differently. That's valuable.</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" ht="60" customHeight="1">
+          <t>Yes, absolutely — unfinished is completely fine to share. Show what you built, show where you got to, and be honest about what you ran out of time for. The most interesting conversations in a show-and-tell often come from "here's where it broke" or "here's what we'd do next," not from polished demos. What you learned from building it matters as much as what you shipped.</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="80" customHeight="1">
       <c r="A33" s="4" t="inlineStr"/>
       <c r="B33" s="5" t="inlineStr">
         <is>
@@ -997,12 +949,10 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>What you built and why. What surprised you. What disappointed you. One thing you'd do differently. You don't need a polished answer — honest reflection is more useful than a confident pitch.</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="n">
-        <v>26</v>
-      </c>
+          <t>Come ready to show what you made — even if it is rough — and say one honest thing about where AI genuinely helped and one place where it disappointed or surprised you. The most useful debriefs are specific: "it kept hallucinating the third step" or "it got us to a working version in 20 minutes but we had to rewrite all the copy" lands better than "it was pretty good." If you had to take the wheel and correct it, say so — that is actually the interesting data. And if you ran out of time or changed direction halfway through, that is worth sharing too. The point is not to present a polished product; it is to have a real point of view.</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -1014,7 +964,7 @@
       <c r="C34" s="3" t="inlineStr"/>
       <c r="D34" s="3" t="inlineStr"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="80" customHeight="1">
       <c r="A35" s="4" t="inlineStr"/>
       <c r="B35" s="5" t="inlineStr">
         <is>
@@ -1023,14 +973,12 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>That's normal. The range of experience in the room is wide by design. Ask a facilitator or the AI Day Guide agent for a concrete next move. The only thing to avoid is waiting.</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="36" ht="60" customHeight="1">
+          <t>Everyone feels this at some point today — the people who look like they know what they're doing mostly just started with something small and kept going. You are not behind. The only thing that matters right now is picking something to build, however small, and starting in the next five minutes. Tell me: are you a researcher or a designer? That one answer will tell me exactly what move to suggest next.</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36" ht="80" customHeight="1">
       <c r="A36" s="8" t="inlineStr"/>
       <c r="B36" s="9" t="inlineStr">
         <is>
@@ -1039,14 +987,12 @@
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>No. There are useful starting points — pick an idea, combine it with an object, start within five minutes — but the path from there is yours. There is no wrong output.</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="37" ht="60" customHeight="1">
+          <t>There is no right way — that is genuinely true, not just reassuring. The only thing that matters is that you end the day with something you made and a real opinion about how it went. Some people will write a spec. Some will build a working tool. Some will make a prototype that breaks in interesting ways. All of those are valid outputs. The question worth asking yourself is not "am I doing this right" but "am I actually making something, or am I still planning to?"</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37" ht="80" customHeight="1">
       <c r="A37" s="4" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
@@ -1055,14 +1001,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Start anyway. Bad ideas become interesting once you try to build them. The act of building is how you find out what the idea actually is.</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="38" ht="60" customHeight="1">
+          <t>There is no bad idea today — there are only ideas you haven't started yet. The point isn't to land on something brilliant before you begin; it's to discover what's interesting by making something. A "bad" idea often turns into a good one the moment you try to build it and hit the first unexpected wall. Pick the seed and object that made you even slightly curious, commit to it for thirty minutes, and see what happens. You can always pivot — but you can't learn anything from an idea you're still only thinking about.</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38" ht="80" customHeight="1">
       <c r="A38" s="8" t="inlineStr"/>
       <c r="B38" s="9" t="inlineStr">
         <is>
@@ -1071,15 +1015,13 @@
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>A genuine point of view on building with AI — what it's good at, where it falls short, what surprised you, and what you'd do differently. That opinion is the output, regardless of what you made.</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="n">
-        <v>30</v>
-      </c>
+          <t>A real point of view — not a theoretical one. By the end of today you should be able to say, from direct experience, where AI actually helps you think and build, and where it flatters you into thinking it's doing more than it is. The artifact you make is almost secondary; what matters is that you got your hands on something and formed an honest opinion. Take that opinion back to your team, your work, your next project — that's the thing that lasts beyond today.</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D38"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>